<commit_message>
Add changes to TestData. xlsx file.
</commit_message>
<xml_diff>
--- a/TDD/TestData.xlsx
+++ b/TDD/TestData.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Claude\Printup project\TDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFCC3C87-C1B1-43AB-908D-CABDCCC809C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D18D05-7585-4B43-ACC9-DC6402396C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15135" yWindow="8985" windowWidth="23595" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9150" yWindow="4185" windowWidth="27465" windowHeight="16110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="161">
   <si>
     <t>ClientInfoFlow</t>
   </si>
@@ -451,40 +451,58 @@
     <t>Type</t>
   </si>
   <si>
-    <t>Add_layer</t>
-  </si>
-  <si>
-    <t>רקע לבן</t>
-  </si>
-  <si>
-    <t>חיתוך</t>
-  </si>
-  <si>
-    <t>צבע</t>
-  </si>
-  <si>
-    <t>הדפסה</t>
-  </si>
-  <si>
-    <t>גוון לבן</t>
-  </si>
-  <si>
-    <t>רקע שחור</t>
-  </si>
-  <si>
-    <t>גוון שחור</t>
-  </si>
-  <si>
-    <t>צלבים</t>
-  </si>
-  <si>
-    <t>תצוגה</t>
-  </si>
-  <si>
-    <t>טקסט</t>
-  </si>
-  <si>
-    <t>בתוך אלמנט</t>
+    <t>editor_name</t>
+  </si>
+  <si>
+    <t>Orly Shalev</t>
+  </si>
+  <si>
+    <t>Yossi Cohen</t>
+  </si>
+  <si>
+    <t>Michal Levi</t>
+  </si>
+  <si>
+    <t>Rotem Sharvit</t>
+  </si>
+  <si>
+    <t>Dana Abraham</t>
+  </si>
+  <si>
+    <t>צבע,צבע</t>
+  </si>
+  <si>
+    <t>צורני,CNC,צמוד</t>
+  </si>
+  <si>
+    <t>index</t>
+  </si>
+  <si>
+    <t>הדפסה,הדפסה</t>
+  </si>
+  <si>
+    <t>חיתוך,חיתוך</t>
+  </si>
+  <si>
+    <t>צלבים,צלבים</t>
+  </si>
+  <si>
+    <t>טקסט,טקסט</t>
+  </si>
+  <si>
+    <t>הדפסה,חיתוך</t>
+  </si>
+  <si>
+    <t>צבע,גוון לבן</t>
+  </si>
+  <si>
+    <t>צבע,גוון שחור</t>
+  </si>
+  <si>
+    <t>צורני,גוון אפור</t>
+  </si>
+  <si>
+    <t>Material_path</t>
   </si>
 </sst>
 </file>
@@ -874,15 +892,18 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -891,15 +912,18 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>10</v>
       </c>
     </row>
@@ -908,15 +932,18 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>14</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>15</v>
       </c>
     </row>
@@ -925,15 +952,18 @@
         <v>16</v>
       </c>
       <c r="B5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -942,15 +972,18 @@
         <v>21</v>
       </c>
       <c r="B6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>25</v>
       </c>
     </row>
@@ -959,15 +992,18 @@
         <v>26</v>
       </c>
       <c r="B7" t="s">
+        <v>147</v>
+      </c>
+      <c r="C7" t="s">
         <v>27</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>28</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>29</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1305,6 +1341,9 @@
       <c r="H23" t="s">
         <v>105</v>
       </c>
+      <c r="I23" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
@@ -1331,6 +1370,9 @@
       <c r="H24" t="s">
         <v>71</v>
       </c>
+      <c r="I24" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -1357,6 +1399,9 @@
       <c r="H25" t="s">
         <v>71</v>
       </c>
+      <c r="I25" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
@@ -1383,6 +1428,9 @@
       <c r="H26" t="s">
         <v>77</v>
       </c>
+      <c r="I26" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1409,6 +1457,9 @@
       <c r="H27" t="s">
         <v>71</v>
       </c>
+      <c r="I27" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
@@ -1435,6 +1486,9 @@
       <c r="H28" t="s">
         <v>77</v>
       </c>
+      <c r="I28" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1449,10 +1503,10 @@
         <v>141</v>
       </c>
       <c r="C30" t="s">
+        <v>151</v>
+      </c>
+      <c r="D30" t="s">
         <v>142</v>
-      </c>
-      <c r="D30" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -1460,13 +1514,13 @@
         <v>106</v>
       </c>
       <c r="B31" t="s">
-        <v>146</v>
-      </c>
-      <c r="C31" t="s">
-        <v>147</v>
+        <v>149</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
       </c>
       <c r="D31" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -1474,13 +1528,13 @@
         <v>112</v>
       </c>
       <c r="B32" t="s">
-        <v>144</v>
-      </c>
-      <c r="C32" t="s">
-        <v>145</v>
+        <v>150</v>
+      </c>
+      <c r="C32">
+        <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -1488,13 +1542,13 @@
         <v>118</v>
       </c>
       <c r="B33" t="s">
-        <v>148</v>
-      </c>
-      <c r="C33" t="s">
-        <v>151</v>
+        <v>157</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1502,13 +1556,13 @@
         <v>125</v>
       </c>
       <c r="B34" t="s">
-        <v>149</v>
-      </c>
-      <c r="C34" t="s">
-        <v>152</v>
+        <v>158</v>
+      </c>
+      <c r="C34">
+        <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1516,22 +1570,22 @@
         <v>132</v>
       </c>
       <c r="B35" t="s">
-        <v>150</v>
-      </c>
-      <c r="C35" t="s">
-        <v>153</v>
+        <v>159</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="C4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="C5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="C7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="C10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="C11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="C12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
@@ -1540,7 +1594,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I15 A22:I22" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I1 A22:I22 A8:I15 A2:A3 G2:I7" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add changes in the TestData.xlsx file.
</commit_message>
<xml_diff>
--- a/TDD/TestData.xlsx
+++ b/TDD/TestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Claude\Printup project\TDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D18D05-7585-4B43-ACC9-DC6402396C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A778AA-CD9A-465D-A316-229557EFB9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9150" yWindow="4185" windowWidth="27465" windowHeight="16110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3405" yWindow="4740" windowWidth="27465" windowHeight="16110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TestData" sheetId="1" r:id="rId1"/>
@@ -28,6 +28,9 @@
     <t>name_surname</t>
   </si>
   <si>
+    <t>editor_name</t>
+  </si>
+  <si>
     <t>main_phone_number</t>
   </si>
   <si>
@@ -43,6 +46,9 @@
     <t>אורלי שלו</t>
   </si>
   <si>
+    <t>Orly Shalev</t>
+  </si>
+  <si>
     <t>0542222222- yes</t>
   </si>
   <si>
@@ -58,6 +64,9 @@
     <t>יוסי כהן</t>
   </si>
   <si>
+    <t>Yossi Cohen</t>
+  </si>
+  <si>
     <t>0547891234 - no</t>
   </si>
   <si>
@@ -73,6 +82,9 @@
     <t>מיכל לוי</t>
   </si>
   <si>
+    <t>Michal Levi</t>
+  </si>
+  <si>
     <t>0523456789 - yes</t>
   </si>
   <si>
@@ -88,6 +100,9 @@
     <t>דנה אברהם</t>
   </si>
   <si>
+    <t>Dana Abraham</t>
+  </si>
+  <si>
     <t>0509876543 - no</t>
   </si>
   <si>
@@ -103,6 +118,9 @@
     <t>רותם שרביט</t>
   </si>
   <si>
+    <t>Rotem Sharvit</t>
+  </si>
+  <si>
     <t>0582345678 - yes</t>
   </si>
   <si>
@@ -205,6 +223,9 @@
     <t>ProjectInfoFlow</t>
   </si>
   <si>
+    <t>Project_path</t>
+  </si>
+  <si>
     <t>Project_name</t>
   </si>
   <si>
@@ -226,6 +247,9 @@
     <t>Status_condition</t>
   </si>
   <si>
+    <t>Materials\1695195183wooden-texture.svg</t>
+  </si>
+  <si>
     <t>פריסת גיליונות</t>
   </si>
   <si>
@@ -241,9 +265,15 @@
     <t>רגיל</t>
   </si>
   <si>
+    <t>ממתין אישור לקוח</t>
+  </si>
+  <si>
     <t>לוודא מרווחים של 4 מ"מ בין אלמנטים</t>
   </si>
   <si>
+    <t>Materials\BackgroundPattern237Colour5.svg</t>
+  </si>
+  <si>
     <t>חיתוך צורני</t>
   </si>
   <si>
@@ -259,12 +289,15 @@
     <t>דחוף</t>
   </si>
   <si>
-    <t>ממתין אישור לקוח</t>
+    <t>הקפאה/בהמתנה</t>
   </si>
   <si>
     <t>חיתוך כרסום בלבד, לא קווי</t>
   </si>
   <si>
+    <t>Materials\FruitPattern2.svg</t>
+  </si>
+  <si>
     <t>הדפסת שכבות</t>
   </si>
   <si>
@@ -277,12 +310,15 @@
     <t>בהול</t>
   </si>
   <si>
-    <t>הקפאה/בהמתנה</t>
+    <t>בוטל</t>
   </si>
   <si>
     <t>שכבת לבן ב-50% שקיפות לבדיקה</t>
   </si>
   <si>
+    <t>Materials\texturelegno.svg</t>
+  </si>
+  <si>
     <t>סידור לוחות</t>
   </si>
   <si>
@@ -292,12 +328,15 @@
     <t>8.4.2026</t>
   </si>
   <si>
-    <t>בוטל</t>
+    <t>תקלה/תיקון</t>
   </si>
   <si>
     <t>הלקוח ביקש כיוון אנכי בלבד</t>
   </si>
   <si>
+    <t>Materials\Wooden-texture-geometry-seamless-pattern-remix.svg</t>
+  </si>
+  <si>
     <t>ריצת דפוס</t>
   </si>
   <si>
@@ -307,7 +346,7 @@
     <t>17.4.2026</t>
   </si>
   <si>
-    <t>תקלה/תיקון</t>
+    <t>ייצור חוזר</t>
   </si>
   <si>
     <t>דחוף - לתאם אישור לקוח לפני הדפסה</t>
@@ -340,7 +379,7 @@
     <t>Keep_in_system</t>
   </si>
   <si>
-    <t>Materials\1695195183wooden-texture.svg</t>
+    <t>Material_path</t>
   </si>
   <si>
     <t>פרספקס</t>
@@ -352,157 +391,118 @@
     <t>שקוף</t>
   </si>
   <si>
+    <t>פולט אור</t>
+  </si>
+  <si>
+    <t>YULI DESIGN</t>
+  </si>
+  <si>
+    <t>פרספקס לבן מבריק</t>
+  </si>
+  <si>
+    <t>PVC</t>
+  </si>
+  <si>
+    <t>שחור</t>
+  </si>
+  <si>
+    <t>מלוטש</t>
+  </si>
+  <si>
+    <t>רשימה B</t>
+  </si>
+  <si>
+    <t>ACM כסוף</t>
+  </si>
+  <si>
+    <t>אלומיניום</t>
+  </si>
+  <si>
+    <t>כסף</t>
+  </si>
+  <si>
+    <t>מט</t>
+  </si>
+  <si>
+    <t>אט</t>
+  </si>
+  <si>
+    <t>קטגוריה A</t>
+  </si>
+  <si>
+    <t>פולט אור שחור</t>
+  </si>
+  <si>
+    <t>פוליפלסט</t>
+  </si>
+  <si>
+    <t>זהב</t>
+  </si>
+  <si>
+    <t>מבריק</t>
+  </si>
+  <si>
+    <t>לפי חומר</t>
+  </si>
+  <si>
+    <t>פרספקס שקוף 6 מ"מ</t>
+  </si>
+  <si>
+    <t>אקריל</t>
+  </si>
+  <si>
+    <t>חלבי</t>
+  </si>
+  <si>
     <t>Yuli design</t>
   </si>
   <si>
-    <t>פרספקס לבן מבריק</t>
-  </si>
-  <si>
-    <t>Materials\BackgroundPattern237Colour5.svg</t>
-  </si>
-  <si>
-    <t>PVC</t>
-  </si>
-  <si>
-    <t>שחור</t>
-  </si>
-  <si>
-    <t>פולט אור</t>
-  </si>
-  <si>
-    <t>רשימה B</t>
-  </si>
-  <si>
-    <t>ACM כסוף</t>
-  </si>
-  <si>
-    <t>Materials\FruitPattern2.svg</t>
-  </si>
-  <si>
-    <t>אלומיניום</t>
-  </si>
-  <si>
-    <t>כסף</t>
-  </si>
-  <si>
-    <t>מט</t>
-  </si>
-  <si>
-    <t>מלוטש</t>
-  </si>
-  <si>
-    <t>קטוגריה A</t>
-  </si>
-  <si>
-    <t>פולט אור שחור</t>
-  </si>
-  <si>
-    <t>Materials\texturelegno.svg</t>
-  </si>
-  <si>
-    <t>פוליפלסט</t>
-  </si>
-  <si>
-    <t>זהב</t>
-  </si>
-  <si>
-    <t>מבריק</t>
-  </si>
-  <si>
-    <t>אט</t>
-  </si>
-  <si>
-    <t>לפי החומר</t>
-  </si>
-  <si>
-    <t>פרספקס שקוף 6 מ"מ</t>
-  </si>
-  <si>
-    <t>Materials\Wooden-texture-geometry-seamless-pattern-remix.svg</t>
-  </si>
-  <si>
-    <t>אקריל</t>
-  </si>
-  <si>
-    <t>חלבי</t>
-  </si>
-  <si>
     <t>מדבקת ויניל מט</t>
   </si>
   <si>
-    <t>YULI DESIGN</t>
-  </si>
-  <si>
-    <t>ייצור חוזר</t>
-  </si>
-  <si>
     <t>LayersInfoFlow</t>
   </si>
   <si>
     <t>Layers_path</t>
   </si>
   <si>
-    <t>Project_path</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
+    <t>index</t>
+  </si>
+  <si>
     <t>Type</t>
   </si>
   <si>
-    <t>editor_name</t>
-  </si>
-  <si>
-    <t>Orly Shalev</t>
-  </si>
-  <si>
-    <t>Yossi Cohen</t>
-  </si>
-  <si>
-    <t>Michal Levi</t>
-  </si>
-  <si>
-    <t>Rotem Sharvit</t>
-  </si>
-  <si>
-    <t>Dana Abraham</t>
-  </si>
-  <si>
     <t>צבע,צבע</t>
   </si>
   <si>
+    <t>הדפסה,הדפסה</t>
+  </si>
+  <si>
     <t>צורני,CNC,צמוד</t>
   </si>
   <si>
-    <t>index</t>
-  </si>
-  <si>
-    <t>הדפסה,הדפסה</t>
-  </si>
-  <si>
     <t>חיתוך,חיתוך</t>
   </si>
   <si>
+    <t>צבע,גוון לבן</t>
+  </si>
+  <si>
     <t>צלבים,צלבים</t>
   </si>
   <si>
+    <t>צבע,גוון שחור</t>
+  </si>
+  <si>
     <t>טקסט,טקסט</t>
   </si>
   <si>
+    <t>צורני,גוון אפור</t>
+  </si>
+  <si>
     <t>הדפסה,חיתוך</t>
-  </si>
-  <si>
-    <t>צבע,גוון לבן</t>
-  </si>
-  <si>
-    <t>צבע,גוון שחור</t>
-  </si>
-  <si>
-    <t>צורני,גוון אפור</t>
-  </si>
-  <si>
-    <t>Material_path</t>
   </si>
 </sst>
 </file>
@@ -892,629 +892,629 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>145</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>146</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>148</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>147</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="C11" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B14" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D14" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>140</v>
+        <v>67</v>
       </c>
       <c r="B16" t="s">
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="E16" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F16" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="G16" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H16" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I16" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="J16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="B17" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="E17" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F17" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="G17" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H17">
         <v>0.33333333333333331</v>
       </c>
       <c r="I17" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J17" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="B18" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E18" t="s">
-        <v>76</v>
+        <v>86</v>
       </c>
       <c r="F18" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="G18" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H18">
         <v>0.4375</v>
       </c>
       <c r="I18" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="J18" t="s">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="D19" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
       <c r="F19" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="G19" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="H19">
         <v>0.54166666666666663</v>
       </c>
       <c r="I19" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="J19" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
+        <v>99</v>
+      </c>
+      <c r="D20" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" t="s">
+        <v>101</v>
+      </c>
+      <c r="F20" t="s">
         <v>87</v>
       </c>
-      <c r="D20" t="s">
-        <v>88</v>
-      </c>
-      <c r="E20" t="s">
-        <v>89</v>
-      </c>
-      <c r="F20" t="s">
-        <v>77</v>
-      </c>
       <c r="G20" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="H20">
         <v>0.64583333333333337</v>
       </c>
       <c r="I20" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="J20" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="D21" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="E21" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="F21" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="G21" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H21">
         <v>0.375</v>
       </c>
       <c r="I21" t="s">
-        <v>137</v>
+        <v>108</v>
       </c>
       <c r="J21" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="B23" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="C23" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="D23" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="E23" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="F23" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="G23" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="H23" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="I23" t="s">
-        <v>160</v>
+        <v>119</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="B24">
         <v>8</v>
       </c>
       <c r="C24" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="E24" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="F24" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="G24" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="H24" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I24" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="B25">
         <v>4</v>
       </c>
       <c r="C25" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="D25" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E25" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="F25" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="G25" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="H25" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I25" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>119</v>
+        <v>131</v>
       </c>
       <c r="B26">
         <v>6</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>132</v>
       </c>
       <c r="D26" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="E26" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F26" t="s">
-        <v>123</v>
+        <v>135</v>
       </c>
       <c r="G26" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="H26" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I26" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="B27">
         <v>6</v>
       </c>
       <c r="C27" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="D27" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="E27" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="F27" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="G27" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="H27" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="I27" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="B28">
         <v>2</v>
       </c>
       <c r="C28" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="D28" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="F28" t="s">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="G28" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="H28" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I28" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B30" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D30" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C31">
         <v>0</v>
@@ -1525,49 +1525,49 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="B32" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C32">
         <v>0</v>
       </c>
       <c r="D32" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
       <c r="B33" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C33">
         <v>1</v>
       </c>
       <c r="D33" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="B34" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C34">
         <v>2</v>
       </c>
       <c r="D34" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>132</v>
+        <v>104</v>
       </c>
       <c r="B35" t="s">
         <v>159</v>
@@ -1576,7 +1576,7 @@
         <v>0</v>
       </c>
       <c r="D35" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -1594,7 +1594,7 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I1 A22:I22 A8:I15 A2:A3 G2:I7" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J22 A24:J25 A23:E23 G23:J23 A27:J27 A26:G26 I26:J26 A29:J35 A28:G28 I28:J28" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>